<commit_message>
docs(literature): full-text analysis notes 02 and 03
Note 02 covers the framework/environment/demand reading of the full-text set;
note 03 extracts RL implementation details from the seven RL papers against a
fixed eight-question frame (policy, decision variables, state transition,
reward, Q update, Q representation, agent definition). Both supersede the
single fulltext_framework_env_demand_analysis.md output, which is removed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/literature_analysis/outputs/screening_results.xlsx
+++ b/literature_analysis/outputs/screening_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xp2239\Desktop\Research_RoadRestoration\literature_analysis\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED3D0C1D-2E53-4841-B887-BAA0A3E4F687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D78A39D-9D6A-49B6-837A-E7F1606BFB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{31C09037-5F22-428F-B1EA-D7EFECE65488}"/>
   </bookViews>
@@ -17021,7 +17021,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -17261,7 +17261,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -18126,7 +18126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -18949,7 +18949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>27</v>
       </c>
@@ -19201,7 +19201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>30</v>
       </c>
@@ -19464,7 +19464,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="34" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>35</v>
       </c>
@@ -20277,7 +20277,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="46" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>49</v>
       </c>
@@ -20357,7 +20357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>50</v>
       </c>
@@ -20984,7 +20984,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="56" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>60</v>
       </c>
@@ -21401,7 +21401,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="62" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>68</v>
       </c>
@@ -23174,7 +23174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>98</v>
       </c>
@@ -23254,7 +23254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>99</v>
       </c>
@@ -54716,7 +54716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="644" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
+    <row r="644" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A644">
         <v>710</v>
       </c>
@@ -56497,7 +56497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="678" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="678" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A678">
         <v>744</v>
       </c>
@@ -57465,7 +57465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="697" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="697" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A697">
         <v>763</v>
       </c>
@@ -63206,7 +63206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="812" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="812" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A812">
         <v>878</v>
       </c>
@@ -64061,7 +64061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="827" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="827" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A827">
         <v>893</v>
       </c>
@@ -65136,7 +65136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="847" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="847" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A847">
         <v>913</v>
       </c>
@@ -70767,7 +70767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="967" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="967" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A967">
         <v>1033</v>
       </c>
@@ -70885,7 +70885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="969" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="969" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A969">
         <v>1035</v>
       </c>
@@ -74256,7 +74256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1033" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1033" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A1033">
         <v>1100</v>
       </c>
@@ -74333,7 +74333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1034" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1034" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A1034">
         <v>1101</v>
       </c>
@@ -74701,7 +74701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1041" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1041" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A1041">
         <v>1108</v>
       </c>
@@ -94057,10 +94057,22 @@
         <filter val="TRUE"/>
       </filters>
     </filterColumn>
-    <filterColumn colId="20">
+    <filterColumn colId="17">
       <filters>
-        <filter val="dynamic/time-varying-demand"/>
+        <filter val="network-flow/capacity"/>
         <filter val="uncertain"/>
+        <filter val="user-equilibrium"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="18">
+      <filters>
+        <filter val="reinforcement-learning/DRL"/>
+        <filter val="reinforcement-learning/DRL; exact/MILP/math-programming"/>
+        <filter val="reinforcement-learning/DRL; graph-neural-network/GNN"/>
+        <filter val="reinforcement-learning/DRL; graph-neural-network/GNN; learn+optimize-hybrid/warmstart-pretraining"/>
+        <filter val="reinforcement-learning/DRL; heuristic/metaheuristic/GA"/>
+        <filter val="reinforcement-learning/DRL; learn+optimize-hybrid/warmstart-pretraining; exact/MILP/math-programming"/>
+        <filter val="reinforcement-learning/DRL; simulation-optimization"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
docs(literature): rename the full-text notes and extend the RL one
The two notes are retitled to name their subject rather than their provenance,
so 02-fulltext_analysis becomes 02-dynamic_demand and
03-RL_implementation_details becomes 03-reinforcement_learning. Note 03 also
grows by a further pass over the RL set. The screening workbooks are refreshed
to match.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/literature_analysis/outputs/screening_results.xlsx
+++ b/literature_analysis/outputs/screening_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xp2239\Desktop\Research_RoadRestoration\literature_analysis\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D78A39D-9D6A-49B6-837A-E7F1606BFB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DFF60AF-C9DA-4179-9A8A-1BBADF738E7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{31C09037-5F22-428F-B1EA-D7EFECE65488}"/>
   </bookViews>
@@ -16549,9 +16549,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -16932,6 +16933,7 @@
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="29" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" customWidth="1"/>
     <col min="19" max="19" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -17021,83 +17023,83 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="2" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="2">
         <v>2025</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="G2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" t="b">
-        <v>0</v>
-      </c>
-      <c r="I2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="N2" t="s">
+      <c r="N2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O2" t="b">
+      <c r="O2" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="s">
+      <c r="P2" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R2" t="s">
+      <c r="R2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="S2" t="s">
+      <c r="S2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T2" t="s">
+      <c r="T2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U2" t="s">
+      <c r="U2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V2" t="s">
+      <c r="V2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X2">
+      <c r="X2" s="2">
         <v>22</v>
       </c>
-      <c r="Y2">
+      <c r="Y2" s="2">
         <v>5.5</v>
       </c>
-      <c r="Z2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA2" t="s">
+      <c r="Z2" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AB2" t="b">
+      <c r="AB2" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -17261,83 +17263,83 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A5">
+    <row r="5" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="2">
         <v>2021</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" t="b">
-        <v>0</v>
-      </c>
-      <c r="I5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J5" t="s">
+      <c r="G5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N5" t="s">
+      <c r="N5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O5" t="b">
+      <c r="O5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P5" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="s">
+      <c r="P5" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R5" t="s">
+      <c r="R5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="S5" t="s">
+      <c r="S5" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T5" t="s">
+      <c r="T5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U5" t="s">
+      <c r="U5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V5" t="s">
+      <c r="V5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W5" t="s">
+      <c r="W5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X5">
+      <c r="X5" s="2">
         <v>77</v>
       </c>
-      <c r="Y5">
+      <c r="Y5" s="2">
         <v>11</v>
       </c>
-      <c r="Z5" t="b">
+      <c r="Z5" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AA5" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="AB5" t="b">
+      <c r="AB5" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -18126,83 +18128,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A16">
+    <row r="16" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="2">
         <v>2026</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G16" t="s">
-        <v>32</v>
-      </c>
-      <c r="H16" t="b">
-        <v>0</v>
-      </c>
-      <c r="I16" t="b">
-        <v>0</v>
-      </c>
-      <c r="J16" t="s">
+      <c r="G16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K16" t="s">
+      <c r="K16" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N16" t="s">
+      <c r="N16" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O16" t="b">
+      <c r="O16" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P16" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="s">
+      <c r="P16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R16" t="s">
+      <c r="R16" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="S16" t="s">
+      <c r="S16" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="T16" t="s">
+      <c r="T16" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U16" t="s">
+      <c r="U16" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V16" t="s">
+      <c r="V16" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W16" t="s">
+      <c r="W16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X16">
-        <v>0</v>
-      </c>
-      <c r="Y16">
-        <v>0</v>
-      </c>
-      <c r="Z16" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA16" t="s">
+      <c r="X16" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AB16" t="b">
+      <c r="AB16" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -18949,89 +18951,89 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A27">
+    <row r="27" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
         <v>27</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="2">
         <v>2023</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="G27" t="s">
-        <v>32</v>
-      </c>
-      <c r="H27" t="b">
-        <v>0</v>
-      </c>
-      <c r="I27" t="b">
-        <v>0</v>
-      </c>
-      <c r="J27" t="s">
+      <c r="G27" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K27" t="s">
+      <c r="K27" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="L27" t="s">
+      <c r="L27" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="M27" t="s">
+      <c r="M27" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="N27" t="s">
+      <c r="N27" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O27" t="b">
+      <c r="O27" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P27" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q27" t="s">
+      <c r="P27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R27" t="s">
+      <c r="R27" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="S27" t="s">
+      <c r="S27" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="T27" t="s">
+      <c r="T27" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="U27" t="s">
+      <c r="U27" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="V27" t="s">
+      <c r="V27" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="W27" t="s">
+      <c r="W27" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X27">
+      <c r="X27" s="2">
         <v>3</v>
       </c>
-      <c r="Y27">
+      <c r="Y27" s="2">
         <v>0.8</v>
       </c>
-      <c r="Z27" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA27" t="s">
+      <c r="Z27" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="AB27" t="b">
+      <c r="AB27" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -19201,83 +19203,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A30">
+    <row r="30" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
         <v>30</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="2">
         <v>2022</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="G30" t="s">
-        <v>32</v>
-      </c>
-      <c r="H30" t="b">
-        <v>0</v>
-      </c>
-      <c r="I30" t="b">
-        <v>0</v>
-      </c>
-      <c r="J30" t="s">
+      <c r="G30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H30" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K30" t="s">
+      <c r="K30" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N30" t="s">
+      <c r="N30" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O30" t="b">
+      <c r="O30" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P30" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="s">
+      <c r="P30" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="R30" t="s">
+      <c r="R30" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="S30" t="s">
+      <c r="S30" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="T30" t="s">
+      <c r="T30" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U30" t="s">
+      <c r="U30" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V30" t="s">
+      <c r="V30" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W30" t="s">
+      <c r="W30" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X30">
+      <c r="X30" s="2">
         <v>27</v>
       </c>
-      <c r="Y30">
+      <c r="Y30" s="2">
         <v>5.4</v>
       </c>
-      <c r="Z30" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA30" t="s">
+      <c r="Z30" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="AB30" t="b">
+      <c r="AB30" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -19464,7 +19466,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="34" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>35</v>
       </c>
@@ -20277,87 +20279,87 @@
         <v>290</v>
       </c>
     </row>
-    <row r="46" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A46">
+    <row r="46" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
         <v>49</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="2">
         <v>2023</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="G46" t="s">
-        <v>32</v>
-      </c>
-      <c r="H46" t="b">
-        <v>0</v>
-      </c>
-      <c r="I46" t="b">
-        <v>0</v>
-      </c>
-      <c r="J46" t="s">
+      <c r="G46" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H46" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J46" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K46" t="s">
+      <c r="K46" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="N46" t="s">
+      <c r="N46" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O46" t="b">
+      <c r="O46" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P46" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q46" t="s">
+      <c r="P46" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R46" t="s">
+      <c r="R46" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="S46" t="s">
+      <c r="S46" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T46" t="s">
+      <c r="T46" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U46" t="s">
+      <c r="U46" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V46" t="s">
+      <c r="V46" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="W46" t="s">
+      <c r="W46" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X46">
+      <c r="X46" s="2">
         <v>9</v>
       </c>
-      <c r="Y46">
+      <c r="Y46" s="2">
         <v>2.2000000000000002</v>
       </c>
-      <c r="Z46" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA46" t="s">
+      <c r="Z46" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA46" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="AB46" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:28" x14ac:dyDescent="0.25">
+      <c r="AB46" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>50</v>
       </c>
@@ -20984,7 +20986,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="56" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>60</v>
       </c>
@@ -21401,83 +21403,83 @@
         <v>216</v>
       </c>
     </row>
-    <row r="62" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A62">
+    <row r="62" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="2">
         <v>68</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="C62">
+      <c r="C62" s="2">
         <v>2026</v>
       </c>
-      <c r="D62" t="s">
+      <c r="D62" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E62" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="F62" t="s">
+      <c r="F62" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="G62" t="s">
-        <v>32</v>
-      </c>
-      <c r="H62" t="b">
-        <v>0</v>
-      </c>
-      <c r="I62" t="b">
-        <v>0</v>
-      </c>
-      <c r="J62" t="s">
+      <c r="G62" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H62" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J62" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K62" t="s">
+      <c r="K62" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N62" t="s">
+      <c r="N62" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O62" t="b">
+      <c r="O62" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P62" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q62" t="s">
+      <c r="P62" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q62" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R62" t="s">
+      <c r="R62" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="S62" t="s">
+      <c r="S62" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="T62" t="s">
+      <c r="T62" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U62" t="s">
+      <c r="U62" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V62" t="s">
+      <c r="V62" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W62" t="s">
+      <c r="W62" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X62">
+      <c r="X62" s="2">
         <v>4</v>
       </c>
-      <c r="Y62">
+      <c r="Y62" s="2">
         <v>2</v>
       </c>
-      <c r="Z62" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA62" t="s">
+      <c r="Z62" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA62" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="AB62" t="b">
+      <c r="AB62" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -23174,7 +23176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>98</v>
       </c>
@@ -23254,83 +23256,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A90">
+    <row r="90" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="2">
         <v>99</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="C90">
+      <c r="C90" s="2">
         <v>2020</v>
       </c>
-      <c r="D90" t="s">
+      <c r="D90" s="2" t="s">
         <v>501</v>
       </c>
-      <c r="E90" t="s">
+      <c r="E90" s="2" t="s">
         <v>502</v>
       </c>
-      <c r="F90" t="s">
+      <c r="F90" s="2" t="s">
         <v>503</v>
       </c>
-      <c r="G90" t="s">
-        <v>32</v>
-      </c>
-      <c r="H90" t="b">
-        <v>0</v>
-      </c>
-      <c r="I90" t="b">
-        <v>0</v>
-      </c>
-      <c r="J90" t="s">
+      <c r="G90" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H90" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I90" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J90" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K90" t="s">
+      <c r="K90" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="N90" t="s">
+      <c r="N90" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O90" t="b">
+      <c r="O90" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P90" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q90" t="s">
+      <c r="P90" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q90" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="R90" t="s">
+      <c r="R90" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="S90" t="s">
+      <c r="S90" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="T90" t="s">
+      <c r="T90" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U90" t="s">
+      <c r="U90" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V90" t="s">
+      <c r="V90" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W90" t="s">
+      <c r="W90" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X90">
+      <c r="X90" s="2">
         <v>40</v>
       </c>
-      <c r="Y90">
+      <c r="Y90" s="2">
         <v>5</v>
       </c>
-      <c r="Z90" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA90" t="s">
+      <c r="Z90" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA90" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="AB90" t="b">
+      <c r="AB90" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -25338,83 +25340,83 @@
         <v>640</v>
       </c>
     </row>
-    <row r="121" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A121">
+    <row r="121" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="2">
         <v>133</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B121" s="2" t="s">
         <v>641</v>
       </c>
-      <c r="C121">
+      <c r="C121" s="2">
         <v>2026</v>
       </c>
-      <c r="D121" t="s">
+      <c r="D121" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E121" t="s">
+      <c r="E121" s="2" t="s">
         <v>642</v>
       </c>
-      <c r="F121" t="s">
+      <c r="F121" s="2" t="s">
         <v>643</v>
       </c>
-      <c r="G121" t="s">
-        <v>32</v>
-      </c>
-      <c r="H121" t="b">
-        <v>0</v>
-      </c>
-      <c r="I121" t="b">
-        <v>0</v>
-      </c>
-      <c r="J121" t="s">
+      <c r="G121" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H121" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I121" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J121" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K121" t="s">
+      <c r="K121" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="N121" t="s">
+      <c r="N121" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O121" t="b">
+      <c r="O121" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P121" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q121" t="s">
+      <c r="P121" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q121" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="R121" t="s">
+      <c r="R121" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="S121" t="s">
+      <c r="S121" s="2" t="s">
         <v>644</v>
       </c>
-      <c r="T121" t="s">
+      <c r="T121" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="U121" t="s">
+      <c r="U121" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="V121" t="s">
+      <c r="V121" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="W121" t="s">
+      <c r="W121" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X121">
-        <v>0</v>
-      </c>
-      <c r="Y121">
-        <v>0</v>
-      </c>
-      <c r="Z121" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA121" t="s">
+      <c r="X121" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y121" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z121" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA121" s="2" t="s">
         <v>645</v>
       </c>
-      <c r="AB121" t="b">
+      <c r="AB121" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -54716,7 +54718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="644" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="644" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
       <c r="A644">
         <v>710</v>
       </c>
@@ -56497,83 +56499,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="678" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A678">
+    <row r="678" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A678" s="2">
         <v>744</v>
       </c>
-      <c r="B678" t="s">
+      <c r="B678" s="2" t="s">
         <v>2691</v>
       </c>
-      <c r="C678">
+      <c r="C678" s="2">
         <v>2007</v>
       </c>
-      <c r="D678" t="s">
+      <c r="D678" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="E678" t="s">
+      <c r="E678" s="2" t="s">
         <v>2692</v>
       </c>
-      <c r="F678" t="s">
+      <c r="F678" s="2" t="s">
         <v>2693</v>
       </c>
-      <c r="G678" t="s">
-        <v>32</v>
-      </c>
-      <c r="H678" t="b">
-        <v>0</v>
-      </c>
-      <c r="I678" t="b">
-        <v>0</v>
-      </c>
-      <c r="J678" t="s">
+      <c r="G678" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H678" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I678" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J678" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K678" t="s">
+      <c r="K678" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N678" t="s">
+      <c r="N678" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O678" t="b">
+      <c r="O678" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P678" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q678" t="s">
+      <c r="P678" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q678" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R678" t="s">
+      <c r="R678" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="S678" t="s">
+      <c r="S678" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T678" t="s">
+      <c r="T678" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U678" t="s">
+      <c r="U678" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V678" t="s">
+      <c r="V678" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W678" t="s">
+      <c r="W678" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X678">
+      <c r="X678" s="2">
         <v>11</v>
       </c>
-      <c r="Y678">
+      <c r="Y678" s="2">
         <v>0.6</v>
       </c>
-      <c r="Z678" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA678" t="s">
+      <c r="Z678" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA678" s="2" t="s">
         <v>2694</v>
       </c>
-      <c r="AB678" t="b">
+      <c r="AB678" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -57465,83 +57467,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="697" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A697">
+    <row r="697" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A697" s="2">
         <v>763</v>
       </c>
-      <c r="B697" t="s">
+      <c r="B697" s="2" t="s">
         <v>2751</v>
       </c>
-      <c r="C697">
+      <c r="C697" s="2">
         <v>2025</v>
       </c>
-      <c r="D697" t="s">
+      <c r="D697" s="2" t="s">
         <v>1497</v>
       </c>
-      <c r="E697" t="s">
+      <c r="E697" s="2" t="s">
         <v>2752</v>
       </c>
-      <c r="F697" t="s">
+      <c r="F697" s="2" t="s">
         <v>2753</v>
       </c>
-      <c r="G697" t="s">
-        <v>32</v>
-      </c>
-      <c r="H697" t="b">
-        <v>0</v>
-      </c>
-      <c r="I697" t="b">
-        <v>0</v>
-      </c>
-      <c r="J697" t="s">
+      <c r="G697" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H697" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I697" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J697" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K697" t="s">
+      <c r="K697" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="N697" t="s">
+      <c r="N697" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O697" t="b">
+      <c r="O697" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P697" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q697" t="s">
+      <c r="P697" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q697" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R697" t="s">
+      <c r="R697" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="S697" t="s">
+      <c r="S697" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T697" t="s">
+      <c r="T697" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U697" t="s">
+      <c r="U697" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V697" t="s">
+      <c r="V697" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W697" t="s">
+      <c r="W697" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X697">
+      <c r="X697" s="2">
         <v>5</v>
       </c>
-      <c r="Y697">
+      <c r="Y697" s="2">
         <v>2.5</v>
       </c>
-      <c r="Z697" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA697" t="s">
+      <c r="Z697" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA697" s="2" t="s">
         <v>2754</v>
       </c>
-      <c r="AB697" t="b">
+      <c r="AB697" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -63206,83 +63208,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="812" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A812">
+    <row r="812" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A812" s="2">
         <v>878</v>
       </c>
-      <c r="B812" t="s">
+      <c r="B812" s="2" t="s">
         <v>3125</v>
       </c>
-      <c r="C812">
+      <c r="C812" s="2">
         <v>2020</v>
       </c>
-      <c r="D812" t="s">
+      <c r="D812" s="2" t="s">
         <v>922</v>
       </c>
-      <c r="E812" t="s">
+      <c r="E812" s="2" t="s">
         <v>3126</v>
       </c>
-      <c r="F812" t="s">
+      <c r="F812" s="2" t="s">
         <v>3127</v>
       </c>
-      <c r="G812" t="s">
-        <v>32</v>
-      </c>
-      <c r="H812" t="b">
-        <v>0</v>
-      </c>
-      <c r="I812" t="b">
-        <v>0</v>
-      </c>
-      <c r="J812" t="s">
+      <c r="G812" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H812" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I812" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J812" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="K812" t="s">
+      <c r="K812" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="N812" t="s">
+      <c r="N812" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O812" t="b">
+      <c r="O812" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P812" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q812" t="s">
+      <c r="P812" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q812" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="R812" t="s">
+      <c r="R812" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="S812" t="s">
+      <c r="S812" s="2" t="s">
         <v>3128</v>
       </c>
-      <c r="T812" t="s">
+      <c r="T812" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="U812" t="s">
+      <c r="U812" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V812" t="s">
+      <c r="V812" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="W812" t="s">
+      <c r="W812" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X812">
+      <c r="X812" s="2">
         <v>31</v>
       </c>
-      <c r="Y812">
+      <c r="Y812" s="2">
         <v>4.4000000000000004</v>
       </c>
-      <c r="Z812" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA812" t="s">
+      <c r="Z812" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA812" s="2" t="s">
         <v>3129</v>
       </c>
-      <c r="AB812" t="b">
+      <c r="AB812" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -64061,83 +64063,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="827" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A827">
+    <row r="827" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A827" s="2">
         <v>893</v>
       </c>
-      <c r="B827" t="s">
+      <c r="B827" s="2" t="s">
         <v>3174</v>
       </c>
-      <c r="C827">
+      <c r="C827" s="2">
         <v>2024</v>
       </c>
-      <c r="D827" t="s">
+      <c r="D827" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E827" t="s">
+      <c r="E827" s="2" t="s">
         <v>3175</v>
       </c>
-      <c r="F827" t="s">
+      <c r="F827" s="2" t="s">
         <v>3176</v>
       </c>
-      <c r="G827" t="s">
-        <v>32</v>
-      </c>
-      <c r="H827" t="b">
-        <v>0</v>
-      </c>
-      <c r="I827" t="b">
-        <v>0</v>
-      </c>
-      <c r="J827" t="s">
+      <c r="G827" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H827" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I827" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J827" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K827" t="s">
+      <c r="K827" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="N827" t="s">
+      <c r="N827" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O827" t="b">
+      <c r="O827" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P827" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q827" t="s">
+      <c r="P827" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q827" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R827" t="s">
+      <c r="R827" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="S827" t="s">
+      <c r="S827" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="T827" t="s">
+      <c r="T827" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U827" t="s">
+      <c r="U827" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V827" t="s">
+      <c r="V827" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="W827" t="s">
+      <c r="W827" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X827">
+      <c r="X827" s="2">
         <v>7</v>
       </c>
-      <c r="Y827">
+      <c r="Y827" s="2">
         <v>2.2999999999999998</v>
       </c>
-      <c r="Z827" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA827" t="s">
+      <c r="Z827" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA827" s="2" t="s">
         <v>3177</v>
       </c>
-      <c r="AB827" t="b">
+      <c r="AB827" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -65136,86 +65138,86 @@
         <v>0</v>
       </c>
     </row>
-    <row r="847" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A847">
+    <row r="847" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A847" s="2">
         <v>913</v>
       </c>
-      <c r="B847" t="s">
+      <c r="B847" s="2" t="s">
         <v>3242</v>
       </c>
-      <c r="C847">
+      <c r="C847" s="2">
         <v>2019</v>
       </c>
-      <c r="D847" t="s">
+      <c r="D847" s="2" t="s">
         <v>768</v>
       </c>
-      <c r="E847" t="s">
+      <c r="E847" s="2" t="s">
         <v>3243</v>
       </c>
-      <c r="F847" t="s">
+      <c r="F847" s="2" t="s">
         <v>3244</v>
       </c>
-      <c r="G847" t="s">
-        <v>32</v>
-      </c>
-      <c r="H847" t="b">
-        <v>0</v>
-      </c>
-      <c r="I847" t="b">
-        <v>0</v>
-      </c>
-      <c r="J847" t="s">
+      <c r="G847" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H847" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I847" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J847" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K847" t="s">
+      <c r="K847" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="L847" t="s">
+      <c r="L847" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="M847" t="s">
+      <c r="M847" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="N847" t="s">
+      <c r="N847" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O847" t="b">
+      <c r="O847" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P847" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q847" t="s">
+      <c r="P847" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q847" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="R847" t="s">
+      <c r="R847" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="S847" t="s">
+      <c r="S847" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="T847" t="s">
+      <c r="T847" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U847" t="s">
+      <c r="U847" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V847" t="s">
+      <c r="V847" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W847" t="s">
+      <c r="W847" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X847">
+      <c r="X847" s="2">
         <v>52</v>
       </c>
-      <c r="Y847">
+      <c r="Y847" s="2">
         <v>6.5</v>
       </c>
-      <c r="Z847" t="b">
+      <c r="Z847" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB847" t="b">
+      <c r="AB847" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -70767,83 +70769,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="967" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A967">
+    <row r="967" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A967" s="2">
         <v>1033</v>
       </c>
-      <c r="B967" t="s">
+      <c r="B967" s="2" t="s">
         <v>3628</v>
       </c>
-      <c r="C967">
+      <c r="C967" s="2">
         <v>2026</v>
       </c>
-      <c r="D967" t="s">
+      <c r="D967" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="E967" t="s">
+      <c r="E967" s="2" t="s">
         <v>3629</v>
       </c>
-      <c r="F967" t="s">
+      <c r="F967" s="2" t="s">
         <v>3630</v>
       </c>
-      <c r="G967" t="s">
-        <v>32</v>
-      </c>
-      <c r="H967" t="b">
-        <v>0</v>
-      </c>
-      <c r="I967" t="b">
-        <v>0</v>
-      </c>
-      <c r="J967" t="s">
+      <c r="G967" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H967" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I967" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J967" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K967" t="s">
+      <c r="K967" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="N967" t="s">
+      <c r="N967" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O967" t="b">
+      <c r="O967" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P967" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q967" t="s">
+      <c r="P967" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q967" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R967" t="s">
+      <c r="R967" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="S967" t="s">
+      <c r="S967" s="2" t="s">
         <v>470</v>
       </c>
-      <c r="T967" t="s">
+      <c r="T967" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U967" t="s">
+      <c r="U967" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V967" t="s">
+      <c r="V967" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W967" t="s">
+      <c r="W967" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X967">
+      <c r="X967" s="2">
         <v>1</v>
       </c>
-      <c r="Y967">
+      <c r="Y967" s="2">
         <v>1</v>
       </c>
-      <c r="Z967" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA967" t="s">
+      <c r="Z967" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA967" s="2" t="s">
         <v>3631</v>
       </c>
-      <c r="AB967" t="b">
+      <c r="AB967" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -70885,83 +70887,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="969" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A969">
+    <row r="969" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A969" s="2">
         <v>1035</v>
       </c>
-      <c r="B969" t="s">
+      <c r="B969" s="2" t="s">
         <v>3636</v>
       </c>
-      <c r="C969">
+      <c r="C969" s="2">
         <v>2018</v>
       </c>
-      <c r="D969" t="s">
+      <c r="D969" s="2" t="s">
         <v>3637</v>
       </c>
-      <c r="E969" t="s">
+      <c r="E969" s="2" t="s">
         <v>3638</v>
       </c>
-      <c r="F969" t="s">
+      <c r="F969" s="2" t="s">
         <v>3639</v>
       </c>
-      <c r="G969" t="s">
-        <v>32</v>
-      </c>
-      <c r="H969" t="b">
-        <v>0</v>
-      </c>
-      <c r="I969" t="b">
-        <v>0</v>
-      </c>
-      <c r="J969" t="s">
+      <c r="G969" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H969" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I969" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J969" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K969" t="s">
+      <c r="K969" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="N969" t="s">
+      <c r="N969" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O969" t="b">
+      <c r="O969" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P969" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q969" t="s">
+      <c r="P969" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q969" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R969" t="s">
+      <c r="R969" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="S969" t="s">
+      <c r="S969" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T969" t="s">
+      <c r="T969" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U969" t="s">
+      <c r="U969" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V969" t="s">
+      <c r="V969" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W969" t="s">
+      <c r="W969" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X969">
+      <c r="X969" s="2">
         <v>99</v>
       </c>
-      <c r="Y969">
+      <c r="Y969" s="2">
         <v>9</v>
       </c>
-      <c r="Z969" t="b">
+      <c r="Z969" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AA969" t="s">
+      <c r="AA969" s="2" t="s">
         <v>3640</v>
       </c>
-      <c r="AB969" t="b">
+      <c r="AB969" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -72191,83 +72193,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="992" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A992">
+    <row r="992" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A992" s="2">
         <v>1059</v>
       </c>
-      <c r="B992" t="s">
+      <c r="B992" s="2" t="s">
         <v>3715</v>
       </c>
-      <c r="C992">
+      <c r="C992" s="2">
         <v>2026</v>
       </c>
-      <c r="D992" t="s">
+      <c r="D992" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="E992" t="s">
+      <c r="E992" s="2" t="s">
         <v>3716</v>
       </c>
-      <c r="F992" t="s">
+      <c r="F992" s="2" t="s">
         <v>3717</v>
       </c>
-      <c r="G992" t="s">
-        <v>32</v>
-      </c>
-      <c r="H992" t="b">
-        <v>0</v>
-      </c>
-      <c r="I992" t="b">
-        <v>0</v>
-      </c>
-      <c r="J992" t="s">
+      <c r="G992" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H992" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I992" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J992" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K992" t="s">
+      <c r="K992" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="N992" t="s">
+      <c r="N992" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O992" t="b">
+      <c r="O992" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P992" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q992" t="s">
+      <c r="P992" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q992" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="R992" t="s">
+      <c r="R992" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="S992" t="s">
+      <c r="S992" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="T992" t="s">
+      <c r="T992" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="U992" t="s">
+      <c r="U992" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V992" t="s">
+      <c r="V992" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W992" t="s">
+      <c r="W992" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X992">
-        <v>0</v>
-      </c>
-      <c r="Y992">
-        <v>0</v>
-      </c>
-      <c r="Z992" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA992" t="s">
+      <c r="X992" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y992" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z992" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA992" s="2" t="s">
         <v>3718</v>
       </c>
-      <c r="AB992" t="b">
+      <c r="AB992" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -74256,157 +74258,157 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1033" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A1033">
+    <row r="1033" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1033" s="2">
         <v>1100</v>
       </c>
-      <c r="B1033" t="s">
+      <c r="B1033" s="2" t="s">
         <v>3847</v>
       </c>
-      <c r="C1033">
+      <c r="C1033" s="2">
         <v>2025</v>
       </c>
-      <c r="D1033" t="s">
+      <c r="D1033" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="E1033" t="s">
+      <c r="E1033" s="2" t="s">
         <v>3848</v>
       </c>
-      <c r="F1033" t="s">
+      <c r="F1033" s="2" t="s">
         <v>3849</v>
       </c>
-      <c r="G1033" t="s">
-        <v>32</v>
-      </c>
-      <c r="H1033" t="b">
-        <v>0</v>
-      </c>
-      <c r="I1033" t="b">
-        <v>0</v>
-      </c>
-      <c r="J1033" t="s">
+      <c r="G1033" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1033" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1033" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J1033" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K1033" t="s">
+      <c r="K1033" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="N1033" t="s">
+      <c r="N1033" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O1033" t="b">
+      <c r="O1033" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P1033" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q1033" t="s">
+      <c r="P1033" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q1033" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R1033" t="s">
+      <c r="R1033" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="S1033" t="s">
+      <c r="S1033" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T1033" t="s">
+      <c r="T1033" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U1033" t="s">
+      <c r="U1033" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V1033" t="s">
+      <c r="V1033" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W1033" t="s">
+      <c r="W1033" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X1033">
+      <c r="X1033" s="2">
         <v>15</v>
       </c>
-      <c r="Y1033">
+      <c r="Y1033" s="2">
         <v>7.5</v>
       </c>
-      <c r="Z1033" t="b">
-        <v>0</v>
-      </c>
-      <c r="AB1033" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="1034" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A1034">
+      <c r="Z1033" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB1033" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1034" s="2">
         <v>1101</v>
       </c>
-      <c r="B1034" t="s">
+      <c r="B1034" s="2" t="s">
         <v>3850</v>
       </c>
-      <c r="C1034">
+      <c r="C1034" s="2">
         <v>2018</v>
       </c>
-      <c r="D1034" t="s">
+      <c r="D1034" s="2" t="s">
         <v>2085</v>
       </c>
-      <c r="E1034" t="s">
+      <c r="E1034" s="2" t="s">
         <v>3851</v>
       </c>
-      <c r="F1034" t="s">
+      <c r="F1034" s="2" t="s">
         <v>3852</v>
       </c>
-      <c r="G1034" t="s">
-        <v>32</v>
-      </c>
-      <c r="H1034" t="b">
-        <v>0</v>
-      </c>
-      <c r="I1034" t="b">
-        <v>0</v>
-      </c>
-      <c r="J1034" t="s">
+      <c r="G1034" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1034" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1034" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J1034" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K1034" t="s">
+      <c r="K1034" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="N1034" t="s">
+      <c r="N1034" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O1034" t="b">
+      <c r="O1034" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P1034" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q1034" t="s">
+      <c r="P1034" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q1034" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R1034" t="s">
+      <c r="R1034" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="S1034" t="s">
-        <v>84</v>
-      </c>
-      <c r="T1034" t="s">
+      <c r="S1034" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="T1034" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U1034" t="s">
+      <c r="U1034" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V1034" t="s">
+      <c r="V1034" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="W1034" t="s">
+      <c r="W1034" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X1034">
+      <c r="X1034" s="2">
         <v>270</v>
       </c>
-      <c r="Y1034">
+      <c r="Y1034" s="2">
         <v>30</v>
       </c>
-      <c r="Z1034" t="b">
+      <c r="Z1034" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="AB1034" t="b">
+      <c r="AB1034" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -74701,83 +74703,83 @@
         <v>0</v>
       </c>
     </row>
-    <row r="1041" spans="1:28" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A1041">
+    <row r="1041" spans="1:28" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1041" s="2">
         <v>1108</v>
       </c>
-      <c r="B1041" t="s">
+      <c r="B1041" s="2" t="s">
         <v>3871</v>
       </c>
-      <c r="C1041">
+      <c r="C1041" s="2">
         <v>2023</v>
       </c>
-      <c r="D1041" t="s">
+      <c r="D1041" s="2" t="s">
         <v>3458</v>
       </c>
-      <c r="E1041" t="s">
+      <c r="E1041" s="2" t="s">
         <v>3872</v>
       </c>
-      <c r="F1041" t="s">
+      <c r="F1041" s="2" t="s">
         <v>3873</v>
       </c>
-      <c r="G1041" t="s">
-        <v>32</v>
-      </c>
-      <c r="H1041" t="b">
-        <v>0</v>
-      </c>
-      <c r="I1041" t="b">
-        <v>0</v>
-      </c>
-      <c r="J1041" t="s">
+      <c r="G1041" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1041" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I1041" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J1041" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="K1041" t="s">
+      <c r="K1041" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="N1041" t="s">
+      <c r="N1041" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="O1041" t="b">
+      <c r="O1041" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="P1041" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q1041" t="s">
+      <c r="P1041" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q1041" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="R1041" t="s">
+      <c r="R1041" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="S1041" t="s">
+      <c r="S1041" s="2" t="s">
         <v>3874</v>
       </c>
-      <c r="T1041" t="s">
+      <c r="T1041" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="U1041" t="s">
+      <c r="U1041" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="V1041" t="s">
+      <c r="V1041" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="W1041" t="s">
+      <c r="W1041" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X1041">
+      <c r="X1041" s="2">
         <v>13</v>
       </c>
-      <c r="Y1041">
+      <c r="Y1041" s="2">
         <v>3.2</v>
       </c>
-      <c r="Z1041" t="b">
-        <v>0</v>
-      </c>
-      <c r="AA1041" t="s">
+      <c r="Z1041" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA1041" s="2" t="s">
         <v>3875</v>
       </c>
-      <c r="AB1041" t="b">
+      <c r="AB1041" s="2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -94057,22 +94059,10 @@
         <filter val="TRUE"/>
       </filters>
     </filterColumn>
-    <filterColumn colId="17">
+    <filterColumn colId="20">
       <filters>
-        <filter val="network-flow/capacity"/>
+        <filter val="dynamic/time-varying-demand"/>
         <filter val="uncertain"/>
-        <filter val="user-equilibrium"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="18">
-      <filters>
-        <filter val="reinforcement-learning/DRL"/>
-        <filter val="reinforcement-learning/DRL; exact/MILP/math-programming"/>
-        <filter val="reinforcement-learning/DRL; graph-neural-network/GNN"/>
-        <filter val="reinforcement-learning/DRL; graph-neural-network/GNN; learn+optimize-hybrid/warmstart-pretraining"/>
-        <filter val="reinforcement-learning/DRL; heuristic/metaheuristic/GA"/>
-        <filter val="reinforcement-learning/DRL; learn+optimize-hybrid/warmstart-pretraining; exact/MILP/math-programming"/>
-        <filter val="reinforcement-learning/DRL; simulation-optimization"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>